<commit_message>
sync: updated all services with latest changes + gitignore for large files
</commit_message>
<xml_diff>
--- a/drywall-takeoff-3d-fbm/Drywall_P_Code_20260122.xlsx
+++ b/drywall-takeoff-3d-fbm/Drywall_P_Code_20260122.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fbmsales-my.sharepoint.com/personal/sean_chang_myfbm_com/Documents/Documents/AI/Drywall/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Debajyoti.R\Downloads\drywall-takeoff-3d-fbm\drywall-takeoff-3d-fbm\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68B1E597-7EFE-4EF5-9AD8-D4A7C9EB9250}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="4680" windowWidth="28800" windowHeight="15345" xr2:uid="{4CEA438F-A519-4CC9-9BAA-5088D567963D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{4CEA438F-A519-4CC9-9BAA-5088D567963D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="333">
   <si>
     <t>PRODUCT_CAT_CODE</t>
   </si>
@@ -1025,6 +1026,15 @@
   </si>
   <si>
     <t>BI - Data Warehouse</t>
+  </si>
+  <si>
+    <t>waste (%)</t>
+  </si>
+  <si>
+    <t>sheet Size (in ft. x ft.)</t>
+  </si>
+  <si>
+    <t>4x8</t>
   </si>
 </sst>
 </file>
@@ -1073,7 +1083,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
   </cellXfs>
@@ -1095,8 +1107,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{15455255-61FB-4001-9C28-A0B831BA6F1E}" name="Table1" displayName="Table1" ref="A1:D201" totalsRowShown="0">
-  <autoFilter ref="A1:D201" xr:uid="{15455255-61FB-4001-9C28-A0B831BA6F1E}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{15455255-61FB-4001-9C28-A0B831BA6F1E}" name="Table1" displayName="Table1" ref="A1:F201" totalsRowShown="0">
+  <autoFilter ref="A1:F201" xr:uid="{15455255-61FB-4001-9C28-A0B831BA6F1E}">
     <filterColumn colId="0">
       <filters>
         <filter val="1010"/>
@@ -1242,11 +1254,13 @@
       </filters>
     </filterColumn>
   </autoFilter>
-  <tableColumns count="4">
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{6BAAC765-778C-464B-A38C-B773BF95BB57}" name="PRODUCT_CAT_CODE"/>
     <tableColumn id="2" xr3:uid="{25E03739-FC0E-4A31-815C-1F25AA3C063B}" name="PRODUCT_CAT_DESC"/>
     <tableColumn id="3" xr3:uid="{81BFF5D6-560F-4B11-B86D-231B442E8C90}" name="user10"/>
     <tableColumn id="4" xr3:uid="{281BD6F9-BF0D-4F87-AB71-04D5966DCD82}" name="user11"/>
+    <tableColumn id="5" xr3:uid="{368C7B3B-FB28-43C8-8F17-F21D23F376A5}" name="waste (%)"/>
+    <tableColumn id="6" xr3:uid="{68CAB50C-818A-49EF-B8DB-8B15951650C1}" name="sheet Size (in ft. x ft.)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1569,16 +1583,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9CC58A4-0625-44C6-98C2-452080F2418B}">
-  <dimension ref="A1:D201"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F201"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" customWidth="1"/>
-    <col min="2" max="2" width="35.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="48.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.453125" customWidth="1"/>
+    <col min="2" max="2" width="35.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" customWidth="1"/>
+    <col min="6" max="6" width="19.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1591,16 +1607,28 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E1" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1010</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" s="2">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1010</v>
       </c>
@@ -1613,8 +1641,14 @@
       <c r="D3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" s="2">
+        <v>10</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1010</v>
       </c>
@@ -1627,8 +1661,14 @@
       <c r="D4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E4" s="2">
+        <v>10</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1010</v>
       </c>
@@ -1641,8 +1681,14 @@
       <c r="D5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E5" s="2">
+        <v>10</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1010</v>
       </c>
@@ -1655,8 +1701,14 @@
       <c r="D6" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E6" s="2">
+        <v>10</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1010</v>
       </c>
@@ -1669,8 +1721,14 @@
       <c r="D7" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E7" s="2">
+        <v>10</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1010</v>
       </c>
@@ -1683,8 +1741,14 @@
       <c r="D8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E8" s="2">
+        <v>10</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1010</v>
       </c>
@@ -1697,8 +1761,14 @@
       <c r="D9" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E9" s="2">
+        <v>10</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>1010</v>
       </c>
@@ -1711,8 +1781,14 @@
       <c r="D10" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E10" s="2">
+        <v>10</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1010</v>
       </c>
@@ -1725,8 +1801,14 @@
       <c r="D11" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E11" s="2">
+        <v>10</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>1010</v>
       </c>
@@ -1739,8 +1821,14 @@
       <c r="D12" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E12" s="2">
+        <v>10</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1010</v>
       </c>
@@ -1753,8 +1841,14 @@
       <c r="D13" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E13" s="2">
+        <v>10</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>1010</v>
       </c>
@@ -1767,8 +1861,14 @@
       <c r="D14" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E14" s="2">
+        <v>10</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1010</v>
       </c>
@@ -1781,8 +1881,14 @@
       <c r="D15" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E15" s="2">
+        <v>10</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>1010</v>
       </c>
@@ -1795,8 +1901,14 @@
       <c r="D16" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E16" s="2">
+        <v>10</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1010</v>
       </c>
@@ -1809,16 +1921,28 @@
       <c r="D17" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E17" s="2">
+        <v>10</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>1015</v>
       </c>
       <c r="B18" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E18" s="2">
+        <v>10</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1015</v>
       </c>
@@ -1831,8 +1955,14 @@
       <c r="D19" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E19" s="2">
+        <v>10</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>1015</v>
       </c>
@@ -1845,8 +1975,14 @@
       <c r="D20" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E20" s="2">
+        <v>10</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>1015</v>
       </c>
@@ -1859,8 +1995,14 @@
       <c r="D21" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E21" s="2">
+        <v>10</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>1015</v>
       </c>
@@ -1873,8 +2015,14 @@
       <c r="D22" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E22" s="2">
+        <v>10</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>1015</v>
       </c>
@@ -1887,8 +2035,14 @@
       <c r="D23" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E23" s="2">
+        <v>10</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>1015</v>
       </c>
@@ -1901,8 +2055,14 @@
       <c r="D24" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E24" s="2">
+        <v>10</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>1015</v>
       </c>
@@ -1915,8 +2075,14 @@
       <c r="D25" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E25" s="2">
+        <v>10</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>1015</v>
       </c>
@@ -1929,8 +2095,14 @@
       <c r="D26" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E26" s="2">
+        <v>10</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>1015</v>
       </c>
@@ -1943,8 +2115,14 @@
       <c r="D27" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E27" s="2">
+        <v>10</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>1015</v>
       </c>
@@ -1957,8 +2135,14 @@
       <c r="D28" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E28" s="2">
+        <v>10</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>1015</v>
       </c>
@@ -1971,8 +2155,14 @@
       <c r="D29" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E29" s="2">
+        <v>10</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>1015</v>
       </c>
@@ -1985,8 +2175,14 @@
       <c r="D30" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E30" s="2">
+        <v>10</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>1015</v>
       </c>
@@ -1999,16 +2195,28 @@
       <c r="D31" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E31" s="2">
+        <v>10</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>1020</v>
       </c>
       <c r="B32" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E32" s="2">
+        <v>10</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>1020</v>
       </c>
@@ -2021,8 +2229,14 @@
       <c r="D33" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E33" s="2">
+        <v>10</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>1020</v>
       </c>
@@ -2035,8 +2249,14 @@
       <c r="D34" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E34" s="2">
+        <v>10</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>1020</v>
       </c>
@@ -2049,8 +2269,14 @@
       <c r="D35" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E35" s="2">
+        <v>10</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>1020</v>
       </c>
@@ -2063,8 +2289,14 @@
       <c r="D36" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E36" s="2">
+        <v>10</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>1020</v>
       </c>
@@ -2077,8 +2309,14 @@
       <c r="D37" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E37" s="2">
+        <v>10</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>1020</v>
       </c>
@@ -2091,8 +2329,14 @@
       <c r="D38" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E38" s="2">
+        <v>10</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>1020</v>
       </c>
@@ -2105,8 +2349,14 @@
       <c r="D39" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E39" s="2">
+        <v>10</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>1020</v>
       </c>
@@ -2119,8 +2369,14 @@
       <c r="D40" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E40" s="2">
+        <v>10</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>1020</v>
       </c>
@@ -2133,8 +2389,14 @@
       <c r="D41" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E41" s="2">
+        <v>10</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>1020</v>
       </c>
@@ -2147,8 +2409,14 @@
       <c r="D42" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E42" s="2">
+        <v>10</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>1020</v>
       </c>
@@ -2161,8 +2429,14 @@
       <c r="D43" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E43" s="2">
+        <v>10</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>1020</v>
       </c>
@@ -2175,8 +2449,14 @@
       <c r="D44" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E44" s="2">
+        <v>10</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>1020</v>
       </c>
@@ -2189,8 +2469,14 @@
       <c r="D45" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E45" s="2">
+        <v>10</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>1020</v>
       </c>
@@ -2203,8 +2489,14 @@
       <c r="D46" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E46" s="2">
+        <v>10</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>1020</v>
       </c>
@@ -2217,8 +2509,14 @@
       <c r="D47" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E47" s="2">
+        <v>10</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>1020</v>
       </c>
@@ -2231,16 +2529,28 @@
       <c r="D48" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E48" s="2">
+        <v>10</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>1025</v>
       </c>
       <c r="B49" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E49" s="2">
+        <v>10</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>1025</v>
       </c>
@@ -2253,8 +2563,14 @@
       <c r="D50" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E50" s="2">
+        <v>10</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>1025</v>
       </c>
@@ -2267,8 +2583,14 @@
       <c r="D51" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E51" s="2">
+        <v>10</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>1025</v>
       </c>
@@ -2281,8 +2603,14 @@
       <c r="D52" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E52" s="2">
+        <v>10</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>1025</v>
       </c>
@@ -2295,8 +2623,14 @@
       <c r="D53" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E53" s="2">
+        <v>10</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>1025</v>
       </c>
@@ -2309,8 +2643,14 @@
       <c r="D54" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E54" s="2">
+        <v>10</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>1025</v>
       </c>
@@ -2323,8 +2663,14 @@
       <c r="D55" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E55" s="2">
+        <v>10</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>1025</v>
       </c>
@@ -2337,8 +2683,14 @@
       <c r="D56" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E56" s="2">
+        <v>10</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>1025</v>
       </c>
@@ -2351,8 +2703,14 @@
       <c r="D57" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E57" s="2">
+        <v>10</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>1025</v>
       </c>
@@ -2365,8 +2723,14 @@
       <c r="D58" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E58" s="2">
+        <v>10</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>1025</v>
       </c>
@@ -2379,8 +2743,14 @@
       <c r="D59" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E59" s="2">
+        <v>10</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>1025</v>
       </c>
@@ -2393,16 +2763,28 @@
       <c r="D60" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E60" s="2">
+        <v>10</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>1030</v>
       </c>
       <c r="B61" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E61" s="2">
+        <v>10</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>1030</v>
       </c>
@@ -2415,8 +2797,14 @@
       <c r="D62" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E62" s="2">
+        <v>10</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>1030</v>
       </c>
@@ -2429,8 +2817,14 @@
       <c r="D63" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E63" s="2">
+        <v>10</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>1030</v>
       </c>
@@ -2443,8 +2837,14 @@
       <c r="D64" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E64" s="2">
+        <v>10</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>1030</v>
       </c>
@@ -2457,8 +2857,14 @@
       <c r="D65" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E65" s="2">
+        <v>10</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>1030</v>
       </c>
@@ -2471,16 +2877,28 @@
       <c r="D66" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="67" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E66" s="2">
+        <v>10</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>1035</v>
       </c>
       <c r="B67" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E67" s="2">
+        <v>10</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>1035</v>
       </c>
@@ -2493,8 +2911,14 @@
       <c r="D68" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E68" s="2">
+        <v>10</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>1035</v>
       </c>
@@ -2507,8 +2931,14 @@
       <c r="D69" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E69" s="2">
+        <v>10</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>1035</v>
       </c>
@@ -2521,8 +2951,14 @@
       <c r="D70" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E70" s="2">
+        <v>10</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>1035</v>
       </c>
@@ -2535,8 +2971,14 @@
       <c r="D71" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E71" s="2">
+        <v>10</v>
+      </c>
+      <c r="F71" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>1035</v>
       </c>
@@ -2549,8 +2991,14 @@
       <c r="D72" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E72" s="2">
+        <v>10</v>
+      </c>
+      <c r="F72" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>1035</v>
       </c>
@@ -2563,8 +3011,14 @@
       <c r="D73" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E73" s="2">
+        <v>10</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>1035</v>
       </c>
@@ -2577,16 +3031,28 @@
       <c r="D74" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="75" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E74" s="2">
+        <v>10</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>1040</v>
       </c>
       <c r="B75" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E75" s="2">
+        <v>10</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>1040</v>
       </c>
@@ -2599,8 +3065,14 @@
       <c r="D76" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E76" s="2">
+        <v>10</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>1040</v>
       </c>
@@ -2613,8 +3085,14 @@
       <c r="D77" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E77" s="2">
+        <v>10</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>1040</v>
       </c>
@@ -2627,8 +3105,14 @@
       <c r="D78" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E78" s="2">
+        <v>10</v>
+      </c>
+      <c r="F78" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>1040</v>
       </c>
@@ -2641,8 +3125,14 @@
       <c r="D79" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E79" s="2">
+        <v>10</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>1040</v>
       </c>
@@ -2655,8 +3145,14 @@
       <c r="D80" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E80" s="2">
+        <v>10</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>1040</v>
       </c>
@@ -2669,8 +3165,14 @@
       <c r="D81" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E81" s="2">
+        <v>10</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>1040</v>
       </c>
@@ -2683,16 +3185,28 @@
       <c r="D82" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="83" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E82" s="2">
+        <v>10</v>
+      </c>
+      <c r="F82" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>1045</v>
       </c>
       <c r="B83" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E83" s="2">
+        <v>10</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>1045</v>
       </c>
@@ -2705,8 +3219,14 @@
       <c r="D84" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E84" s="2">
+        <v>10</v>
+      </c>
+      <c r="F84" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>1045</v>
       </c>
@@ -2719,8 +3239,14 @@
       <c r="D85" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E85" s="2">
+        <v>10</v>
+      </c>
+      <c r="F85" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>1045</v>
       </c>
@@ -2733,8 +3259,14 @@
       <c r="D86" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E86" s="2">
+        <v>10</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>1045</v>
       </c>
@@ -2747,8 +3279,14 @@
       <c r="D87" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E87" s="2">
+        <v>10</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>1045</v>
       </c>
@@ -2761,8 +3299,14 @@
       <c r="D88" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E88" s="2">
+        <v>10</v>
+      </c>
+      <c r="F88" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>1045</v>
       </c>
@@ -2775,8 +3319,14 @@
       <c r="D89" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E89" s="2">
+        <v>10</v>
+      </c>
+      <c r="F89" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>1045</v>
       </c>
@@ -2789,8 +3339,14 @@
       <c r="D90" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E90" s="2">
+        <v>10</v>
+      </c>
+      <c r="F90" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>1045</v>
       </c>
@@ -2803,8 +3359,14 @@
       <c r="D91" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E91" s="2">
+        <v>10</v>
+      </c>
+      <c r="F91" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>1045</v>
       </c>
@@ -2817,8 +3379,14 @@
       <c r="D92" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E92" s="2">
+        <v>10</v>
+      </c>
+      <c r="F92" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>1045</v>
       </c>
@@ -2831,8 +3399,14 @@
       <c r="D93" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E93" s="2">
+        <v>10</v>
+      </c>
+      <c r="F93" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>1045</v>
       </c>
@@ -2845,8 +3419,14 @@
       <c r="D94" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E94" s="2">
+        <v>10</v>
+      </c>
+      <c r="F94" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>1045</v>
       </c>
@@ -2859,8 +3439,14 @@
       <c r="D95" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E95" s="2">
+        <v>10</v>
+      </c>
+      <c r="F95" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>1045</v>
       </c>
@@ -2873,16 +3459,28 @@
       <c r="D96" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="97" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E96" s="2">
+        <v>10</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>1050</v>
       </c>
       <c r="B97" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E97" s="2">
+        <v>10</v>
+      </c>
+      <c r="F97" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>1050</v>
       </c>
@@ -2895,16 +3493,28 @@
       <c r="D98" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="99" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E98" s="2">
+        <v>10</v>
+      </c>
+      <c r="F98" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>1051</v>
       </c>
       <c r="B99" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E99" s="2">
+        <v>10</v>
+      </c>
+      <c r="F99" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>1051</v>
       </c>
@@ -2917,16 +3527,28 @@
       <c r="D100" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E100" s="2">
+        <v>10</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>1052</v>
       </c>
       <c r="B101" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E101" s="2">
+        <v>10</v>
+      </c>
+      <c r="F101" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>1052</v>
       </c>
@@ -2939,16 +3561,28 @@
       <c r="D102" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="103" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E102" s="2">
+        <v>10</v>
+      </c>
+      <c r="F102" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>1060</v>
       </c>
       <c r="B103" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E103" s="2">
+        <v>10</v>
+      </c>
+      <c r="F103" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>1060</v>
       </c>
@@ -2961,8 +3595,14 @@
       <c r="D104" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E104" s="2">
+        <v>10</v>
+      </c>
+      <c r="F104" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>1060</v>
       </c>
@@ -2975,8 +3615,14 @@
       <c r="D105" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E105" s="2">
+        <v>10</v>
+      </c>
+      <c r="F105" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>1060</v>
       </c>
@@ -2989,8 +3635,14 @@
       <c r="D106" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E106" s="2">
+        <v>10</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>1060</v>
       </c>
@@ -3003,16 +3655,28 @@
       <c r="D107" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="108" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E107" s="2">
+        <v>10</v>
+      </c>
+      <c r="F107" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>1070</v>
       </c>
       <c r="B108" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E108" s="2">
+        <v>10</v>
+      </c>
+      <c r="F108" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>1070</v>
       </c>
@@ -3025,8 +3689,14 @@
       <c r="D109" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E109" s="2">
+        <v>10</v>
+      </c>
+      <c r="F109" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>1070</v>
       </c>
@@ -3039,8 +3709,14 @@
       <c r="D110" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E110" s="2">
+        <v>10</v>
+      </c>
+      <c r="F110" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>1070</v>
       </c>
@@ -3053,8 +3729,14 @@
       <c r="D111" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E111" s="2">
+        <v>10</v>
+      </c>
+      <c r="F111" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>1070</v>
       </c>
@@ -3067,8 +3749,14 @@
       <c r="D112" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E112" s="2">
+        <v>10</v>
+      </c>
+      <c r="F112" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>1070</v>
       </c>
@@ -3081,8 +3769,14 @@
       <c r="D113" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E113" s="2">
+        <v>10</v>
+      </c>
+      <c r="F113" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>1070</v>
       </c>
@@ -3095,8 +3789,14 @@
       <c r="D114" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E114" s="2">
+        <v>10</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>1070</v>
       </c>
@@ -3109,16 +3809,28 @@
       <c r="D115" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E115" s="2">
+        <v>10</v>
+      </c>
+      <c r="F115" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>1080</v>
       </c>
       <c r="B116" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E116" s="2">
+        <v>10</v>
+      </c>
+      <c r="F116" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>1080</v>
       </c>
@@ -3131,8 +3843,14 @@
       <c r="D117" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E117" s="2">
+        <v>10</v>
+      </c>
+      <c r="F117" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>1080</v>
       </c>
@@ -3145,8 +3863,14 @@
       <c r="D118" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E118" s="2">
+        <v>10</v>
+      </c>
+      <c r="F118" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>1080</v>
       </c>
@@ -3159,8 +3883,14 @@
       <c r="D119" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E119" s="2">
+        <v>10</v>
+      </c>
+      <c r="F119" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>1080</v>
       </c>
@@ -3173,8 +3903,14 @@
       <c r="D120" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E120" s="2">
+        <v>10</v>
+      </c>
+      <c r="F120" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>1080</v>
       </c>
@@ -3187,8 +3923,14 @@
       <c r="D121" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E121" s="2">
+        <v>10</v>
+      </c>
+      <c r="F121" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>1080</v>
       </c>
@@ -3201,8 +3943,14 @@
       <c r="D122" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E122" s="2">
+        <v>10</v>
+      </c>
+      <c r="F122" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>1080</v>
       </c>
@@ -3215,8 +3963,14 @@
       <c r="D123" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E123" s="2">
+        <v>10</v>
+      </c>
+      <c r="F123" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>1080</v>
       </c>
@@ -3229,16 +3983,28 @@
       <c r="D124" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="125" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E124" s="2">
+        <v>10</v>
+      </c>
+      <c r="F124" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>1090</v>
       </c>
       <c r="B125" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E125" s="2">
+        <v>10</v>
+      </c>
+      <c r="F125" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>1090</v>
       </c>
@@ -3251,8 +4017,14 @@
       <c r="D126" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E126" s="2">
+        <v>10</v>
+      </c>
+      <c r="F126" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>1090</v>
       </c>
@@ -3265,8 +4037,14 @@
       <c r="D127" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E127" s="2">
+        <v>10</v>
+      </c>
+      <c r="F127" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>1090</v>
       </c>
@@ -3279,8 +4057,14 @@
       <c r="D128" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E128" s="2">
+        <v>10</v>
+      </c>
+      <c r="F128" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>1090</v>
       </c>
@@ -3293,8 +4077,14 @@
       <c r="D129" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E129" s="2">
+        <v>10</v>
+      </c>
+      <c r="F129" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>1090</v>
       </c>
@@ -3307,8 +4097,14 @@
       <c r="D130" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E130" s="2">
+        <v>10</v>
+      </c>
+      <c r="F130" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>1090</v>
       </c>
@@ -3321,8 +4117,14 @@
       <c r="D131" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E131" s="2">
+        <v>10</v>
+      </c>
+      <c r="F131" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>1090</v>
       </c>
@@ -3335,8 +4137,14 @@
       <c r="D132" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E132" s="2">
+        <v>10</v>
+      </c>
+      <c r="F132" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>1090</v>
       </c>
@@ -3349,8 +4157,14 @@
       <c r="D133" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E133" s="2">
+        <v>10</v>
+      </c>
+      <c r="F133" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>1090</v>
       </c>
@@ -3363,8 +4177,14 @@
       <c r="D134" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E134" s="2">
+        <v>10</v>
+      </c>
+      <c r="F134" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>1090</v>
       </c>
@@ -3377,8 +4197,14 @@
       <c r="D135" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E135" s="2">
+        <v>10</v>
+      </c>
+      <c r="F135" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>1090</v>
       </c>
@@ -3391,8 +4217,14 @@
       <c r="D136" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E136" s="2">
+        <v>10</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>1090</v>
       </c>
@@ -3405,8 +4237,14 @@
       <c r="D137" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="138" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E137" s="2">
+        <v>10</v>
+      </c>
+      <c r="F137" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>1090</v>
       </c>
@@ -3420,7 +4258,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>1090</v>
       </c>
@@ -3433,8 +4271,14 @@
       <c r="D139" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="140" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E139" s="2">
+        <v>10</v>
+      </c>
+      <c r="F139" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>1097</v>
       </c>
@@ -3442,7 +4286,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="141" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>1097</v>
       </c>
@@ -3456,7 +4300,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="142" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>1098</v>
       </c>
@@ -3464,7 +4308,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="143" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>1098</v>
       </c>
@@ -3478,7 +4322,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="144" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144">
         <v>1099</v>
       </c>
@@ -3486,7 +4330,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="145" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>1099</v>
       </c>
@@ -3500,7 +4344,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A146">
         <v>1099</v>
       </c>
@@ -3513,8 +4357,14 @@
       <c r="D146" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E146" s="2">
+        <v>10</v>
+      </c>
+      <c r="F146" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A147">
         <v>1099</v>
       </c>
@@ -3527,8 +4377,14 @@
       <c r="D147" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E147" s="2">
+        <v>10</v>
+      </c>
+      <c r="F147" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A148">
         <v>1099</v>
       </c>
@@ -3541,8 +4397,14 @@
       <c r="D148" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E148" s="2">
+        <v>10</v>
+      </c>
+      <c r="F148" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A149">
         <v>1099</v>
       </c>
@@ -3555,8 +4417,14 @@
       <c r="D149" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E149" s="2">
+        <v>10</v>
+      </c>
+      <c r="F149" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A150">
         <v>1099</v>
       </c>
@@ -3569,8 +4437,14 @@
       <c r="D150" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E150" s="2">
+        <v>10</v>
+      </c>
+      <c r="F150" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A151">
         <v>1099</v>
       </c>
@@ -3580,8 +4454,14 @@
       <c r="C151" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E151" s="2">
+        <v>10</v>
+      </c>
+      <c r="F151" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A152">
         <v>1099</v>
       </c>
@@ -3594,8 +4474,14 @@
       <c r="D152" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E152" s="2">
+        <v>10</v>
+      </c>
+      <c r="F152" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A153">
         <v>1099</v>
       </c>
@@ -3608,8 +4494,14 @@
       <c r="D153" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E153" s="2">
+        <v>10</v>
+      </c>
+      <c r="F153" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A154">
         <v>1099</v>
       </c>
@@ -3622,8 +4514,14 @@
       <c r="D154" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E154" s="2">
+        <v>10</v>
+      </c>
+      <c r="F154" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A155">
         <v>1099</v>
       </c>
@@ -3636,8 +4534,14 @@
       <c r="D155" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E155" s="2">
+        <v>10</v>
+      </c>
+      <c r="F155" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A156">
         <v>1099</v>
       </c>
@@ -3650,8 +4554,14 @@
       <c r="D156" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E156" s="2">
+        <v>10</v>
+      </c>
+      <c r="F156" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A157">
         <v>1099</v>
       </c>
@@ -3664,8 +4574,14 @@
       <c r="D157" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E157" s="2">
+        <v>10</v>
+      </c>
+      <c r="F157" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A158">
         <v>1099</v>
       </c>
@@ -3678,8 +4594,14 @@
       <c r="D158" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E158" s="2">
+        <v>10</v>
+      </c>
+      <c r="F158" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A159">
         <v>1099</v>
       </c>
@@ -3692,8 +4614,14 @@
       <c r="D159" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E159" s="2">
+        <v>10</v>
+      </c>
+      <c r="F159" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A160">
         <v>1099</v>
       </c>
@@ -3706,8 +4634,14 @@
       <c r="D160" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="161" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E160" s="2">
+        <v>10</v>
+      </c>
+      <c r="F160" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161">
         <v>1099</v>
       </c>
@@ -3721,7 +4655,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A162">
         <v>1099</v>
       </c>
@@ -3734,8 +4668,14 @@
       <c r="D162" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E162" s="2">
+        <v>10</v>
+      </c>
+      <c r="F162" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A163">
         <v>1099</v>
       </c>
@@ -3748,8 +4688,14 @@
       <c r="D163" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="164" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E163" s="2">
+        <v>10</v>
+      </c>
+      <c r="F163" s="2" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164">
         <v>1099</v>
       </c>
@@ -3763,7 +4709,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="165" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>261</v>
       </c>
@@ -3771,7 +4717,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="166" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" t="s">
         <v>263</v>
       </c>
@@ -3779,7 +4725,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="167" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>265</v>
       </c>
@@ -3787,7 +4733,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="168" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>267</v>
       </c>
@@ -3795,7 +4741,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="169" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>269</v>
       </c>
@@ -3803,7 +4749,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="170" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A170" t="s">
         <v>271</v>
       </c>
@@ -3811,7 +4757,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="171" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>273</v>
       </c>
@@ -3819,7 +4765,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="172" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>275</v>
       </c>
@@ -3827,7 +4773,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="173" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>277</v>
       </c>
@@ -3835,7 +4781,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="174" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A174" t="s">
         <v>279</v>
       </c>
@@ -3843,7 +4789,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="175" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" t="s">
         <v>281</v>
       </c>
@@ -3851,7 +4797,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="176" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" t="s">
         <v>283</v>
       </c>
@@ -3859,7 +4805,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="177" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" t="s">
         <v>285</v>
       </c>
@@ -3867,7 +4813,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="178" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" t="s">
         <v>287</v>
       </c>
@@ -3875,7 +4821,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="179" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" t="s">
         <v>289</v>
       </c>
@@ -3883,7 +4829,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="180" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" t="s">
         <v>291</v>
       </c>
@@ -3891,7 +4837,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="181" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" t="s">
         <v>293</v>
       </c>
@@ -3899,7 +4845,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="182" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" t="s">
         <v>295</v>
       </c>
@@ -3907,7 +4853,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="183" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" t="s">
         <v>297</v>
       </c>
@@ -3915,7 +4861,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="184" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" t="s">
         <v>299</v>
       </c>
@@ -3923,7 +4869,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="185" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185" t="s">
         <v>301</v>
       </c>
@@ -3931,7 +4877,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="186" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" t="s">
         <v>303</v>
       </c>
@@ -3939,7 +4885,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="187" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" t="s">
         <v>305</v>
       </c>
@@ -3947,7 +4893,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="188" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A188" t="s">
         <v>307</v>
       </c>
@@ -3955,7 +4901,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="189" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" t="s">
         <v>309</v>
       </c>
@@ -3963,7 +4909,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="190" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190" t="s">
         <v>311</v>
       </c>
@@ -3971,7 +4917,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="191" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191" t="s">
         <v>313</v>
       </c>
@@ -3979,7 +4925,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="192" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192" t="s">
         <v>315</v>
       </c>
@@ -3987,7 +4933,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="193" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A193" t="s">
         <v>317</v>
       </c>
@@ -3995,7 +4941,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="194" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" t="s">
         <v>319</v>
       </c>
@@ -4003,7 +4949,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="195" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" t="s">
         <v>321</v>
       </c>
@@ -4011,7 +4957,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="196" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A196" t="s">
         <v>323</v>
       </c>
@@ -4019,7 +4965,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="197" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197" t="s">
         <v>325</v>
       </c>
@@ -4027,7 +4973,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="198" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A198">
         <v>2011</v>
       </c>
@@ -4035,7 +4981,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="199" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A199">
         <v>2011</v>
       </c>
@@ -4049,7 +4995,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="200" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200">
         <v>2011</v>
       </c>
@@ -4063,7 +5009,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="201" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A201" t="s">
         <v>328</v>
       </c>

</xml_diff>